<commit_message>
feat: Enhance passenger timeline functionality with FTE data and improve UI for flight selection
</commit_message>
<xml_diff>
--- a/data/flight_delay_effect.xlsx
+++ b/data/flight_delay_effect.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9979a6a62ab1ab53/Coding/python_scripts/DAA-Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="11_CA418FE7B924141FDB9A40373AEE2AD6CABFD25E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24292B83-676C-44D5-B431-31DD49C13882}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="11_CA418FE7B924141FDB9A40373AEE2AD6CABFD25E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{308CB891-CA2C-494D-A594-18E29E86AAD7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -194,8 +194,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="168" formatCode="h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="h:mm:ss"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -249,8 +249,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1341,7 +1341,7 @@
         <v>43</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F11">
         <v>13</v>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="S11">
         <f t="shared" si="0"/>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="T11">
         <f t="shared" si="0"/>
@@ -1416,7 +1416,7 @@
         <v>94</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F12">
         <v>23</v>
@@ -1462,7 +1462,7 @@
       </c>
       <c r="S12">
         <f t="shared" si="0"/>
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="T12">
         <f t="shared" si="0"/>
@@ -1491,7 +1491,7 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F13">
         <v>43</v>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="S13">
         <f t="shared" si="0"/>
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="T13">
         <f t="shared" si="0"/>
@@ -1566,7 +1566,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F14">
         <v>94</v>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="S14">
         <f t="shared" si="0"/>
-        <v>-13</v>
+        <v>0</v>
       </c>
       <c r="T14">
         <f t="shared" si="0"/>
@@ -1641,7 +1641,7 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -1662,7 +1662,7 @@
         <v>43</v>
       </c>
       <c r="L15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M15">
         <v>13</v>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="S15">
         <f t="shared" si="0"/>
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="T15">
         <f t="shared" si="0"/>
@@ -1716,7 +1716,7 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -1737,7 +1737,7 @@
         <v>94</v>
       </c>
       <c r="L16">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M16">
         <v>23</v>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="S16">
         <f t="shared" si="0"/>
-        <v>-38</v>
+        <v>0</v>
       </c>
       <c r="T16">
         <f t="shared" si="0"/>
@@ -1791,7 +1791,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1812,7 +1812,7 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M17">
         <v>43</v>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="S17">
         <f t="shared" si="0"/>
-        <v>-89</v>
+        <v>0</v>
       </c>
       <c r="T17">
         <f t="shared" si="0"/>
@@ -1887,7 +1887,7 @@
         <v>0</v>
       </c>
       <c r="L18">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="M18">
         <v>94</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="S18">
         <f t="shared" ref="S18:S23" si="4">L18-E18</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="T18">
         <f t="shared" ref="T18:T23" si="5">M18-F18</f>
@@ -1962,7 +1962,7 @@
         <v>0</v>
       </c>
       <c r="L19">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="M19">
         <v>0</v>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="S19">
         <f t="shared" si="4"/>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="T19">
         <f t="shared" si="5"/>
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="L20">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="M20">
         <v>0</v>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="S20">
         <f t="shared" si="4"/>
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="T20">
         <f t="shared" si="5"/>
@@ -2112,7 +2112,7 @@
         <v>0</v>
       </c>
       <c r="L21">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="M21">
         <v>0</v>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="S21">
         <f t="shared" si="4"/>
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="T21">
         <f t="shared" si="5"/>

</xml_diff>